<commit_message>
4.0 files and model
</commit_message>
<xml_diff>
--- a/InputData/ccs/CCP/CO2 Capture Potentials.xlsx
+++ b/InputData/ccs/CCP/CO2 Capture Potentials.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\ccs\CCP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB242916-3486-4863-B65A-1BC02A5C7437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB7172B8-79FD-4360-98F3-E9249B18DB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="CPPbES" sheetId="12" r:id="rId2"/>
     <sheet name="CPPbI" sheetId="13" r:id="rId3"/>
+    <sheet name="CPPbHS" sheetId="15" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
   <si>
     <t>Source:</t>
   </si>
@@ -313,6 +314,12 @@
   </si>
   <si>
     <t>hydrogen combined cycle</t>
+  </si>
+  <si>
+    <t>natural gas reforming with CCS</t>
+  </si>
+  <si>
+    <t>capture rate</t>
   </si>
 </sst>
 </file>
@@ -1348,4 +1355,38 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D48B9D0-7C8A-4023-B3D1-3CE3C9AF0583}">
+  <sheetPr>
+    <tabColor theme="3"/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="45.42578125" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2">
+        <v>0.85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>